<commit_message>
Aktualizuj wycenę V5 — usuń koszty sprzętu (MacBook i iPady własne dewelopera)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Wycena_Kielich_v5.xlsx
+++ b/Wycena_Kielich_v5.xlsx
@@ -850,7 +850,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Mac wymagany do kompilacji Xcode. 2×iPad do testów P2P (Multipeer wymaga fizycznych urządzeń). Cały pozostały development na symulatorze Xcode.</t>
+          <t>MacBook i iPady — własne, już posiadane przez dewelopera. Brak kosztu sprzętowego dla projektu. Multipeer Connectivity wymaga fizycznych iPadów (symulator nie obsługuje) — pokryte posiadanym sprzętem.</t>
         </is>
       </c>
     </row>
@@ -996,14 +996,14 @@
       </c>
       <c r="D20" s="16" t="inlineStr">
         <is>
-          <t>App Store + TestFlight + dystrybucja komercyjna</t>
+          <t>App Store + TestFlight + dystrybucja komercyjna. Jedyny zewnętrzny koszt — MacBook i iPady posiada developer.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>2× iPad Pro (testy Multipeer P2P)</t>
+          <t>MacBook (kompilacja Xcode)</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
@@ -1013,19 +1013,19 @@
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>5 000 PLN</t>
+          <t>0 PLN</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr">
         <is>
-          <t>Fizyczne urządzenia — Multipeer Connectivity nie działa na symulatorze</t>
+          <t>Developer posiada własny MacBook — brak kosztu</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>Akcesoria (kable, adaptery, hub USB-C)</t>
+          <t>iPady (testy Multipeer P2P)</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
@@ -1035,19 +1035,19 @@
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>300 PLN</t>
+          <t>0 PLN</t>
         </is>
       </c>
       <c r="D22" s="16" t="inlineStr">
         <is>
-          <t>Jednorazowe wyposażenie stanowiska</t>
+          <t>Developer posiada własne iPady — brak kosztu</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="21" t="inlineStr">
         <is>
-          <t>KOSZTY STAŁE (sprzęt + licencje)</t>
+          <t>KOSZTY STAŁE</t>
         </is>
       </c>
       <c r="B23" s="22" t="inlineStr">
@@ -1057,12 +1057,12 @@
       </c>
       <c r="C23" s="23" t="inlineStr">
         <is>
-          <t>5 700 PLN</t>
+          <t>400 PLN/rok</t>
         </is>
       </c>
       <c r="D23" s="24" t="inlineStr">
         <is>
-          <t>Doliczane do robocizny</t>
+          <t>Wyłącznie Apple Developer Account — sprzęt już posiadany</t>
         </is>
       </c>
     </row>
@@ -1077,12 +1077,12 @@
       </c>
       <c r="C24" s="27" t="inlineStr">
         <is>
-          <t>33 650 PLN</t>
+          <t>28 350 PLN</t>
         </is>
       </c>
       <c r="D24" s="28" t="inlineStr">
         <is>
-          <t>Robocizna 27 950 PLN + koszty stałe 5 700 PLN</t>
+          <t>Robocizna 27 950 PLN + Apple Dev 400 PLN</t>
         </is>
       </c>
     </row>
@@ -1835,12 +1835,12 @@
       </c>
       <c r="H5" s="54" t="inlineStr">
         <is>
-          <t>5 700 PLN</t>
+          <t>400 PLN</t>
         </is>
       </c>
       <c r="I5" s="54" t="inlineStr">
         <is>
-          <t>21 300 PLN</t>
+          <t>16 000 PLN</t>
         </is>
       </c>
     </row>
@@ -1880,12 +1880,12 @@
       </c>
       <c r="H6" s="54" t="inlineStr">
         <is>
-          <t>5 700 PLN</t>
+          <t>400 PLN</t>
         </is>
       </c>
       <c r="I6" s="54" t="inlineStr">
         <is>
-          <t>25 800 PLN</t>
+          <t>20 500 PLN</t>
         </is>
       </c>
     </row>
@@ -1925,12 +1925,12 @@
       </c>
       <c r="H7" s="54" t="inlineStr">
         <is>
-          <t>5 700 PLN</t>
+          <t>400 PLN</t>
         </is>
       </c>
       <c r="I7" s="54" t="inlineStr">
         <is>
-          <t>30 100 PLN</t>
+          <t>24 800 PLN</t>
         </is>
       </c>
     </row>
@@ -1966,12 +1966,12 @@
       </c>
       <c r="H8" s="55" t="inlineStr">
         <is>
-          <t>5 701 PLN</t>
+          <t>400 PLN</t>
         </is>
       </c>
       <c r="I8" s="55" t="inlineStr">
         <is>
-          <t>55 151 PLN</t>
+          <t>49 850 PLN</t>
         </is>
       </c>
     </row>
@@ -2007,12 +2007,12 @@
       </c>
       <c r="H9" s="56" t="inlineStr">
         <is>
-          <t>5 700 PLN</t>
+          <t>400 PLN</t>
         </is>
       </c>
       <c r="I9" s="56" t="inlineStr">
         <is>
-          <t>33 650 PLN</t>
+          <t>28 350 PLN</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2162,95 +2162,95 @@
       </c>
       <c r="E4" s="16" t="inlineStr">
         <is>
-          <t>Wymagane do App Store, TestFlight, dystrybucji IPA. Firma lub osoba fizyczna. Rejestracja ~2 tygodnie.</t>
+          <t>Jedyny zewnętrzny koszt. Wymagane do App Store, TestFlight, dystrybucji IPA. Firma lub osoba fizyczna. Rejestracja ~2 tygodnie.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>iPad 1 (Monitor)</t>
+          <t>MacBook (kompilacja Xcode)</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>2 500 PLN</t>
+          <t>0 PLN</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Jednorazowo</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>TAK</t>
+          <t>POSIADANY</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Testowanie wyświetlania Monitor UI + Multipeer (symulator nie obsługuje MC)</t>
+          <t>Developer posiada własny MacBook — brak kosztu dla projektu.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>iPad 2 (Pilot)</t>
+          <t>iPady (testy Multipeer P2P)</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>2 500 PLN</t>
+          <t>0 PLN</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>Jednorazowo</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>TAK</t>
+          <t>POSIADANE</t>
         </is>
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>Testowanie sterowania Pilot UI + połączenia P2P 1:1</t>
+          <t>Developer posiada własne iPady. Multipeer wymaga fizycznych urządzeń (symulator nie obsługuje MC) — pokryte przez posiadany sprzęt.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Akcesoria (kable USB-C, hub, etui)</t>
+          <t>VS Code / .NET SDK / Xcode</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>300 PLN</t>
+          <t>0 PLN</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Jednorazowo</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>TAK</t>
+          <t>DARMOWE</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Kabel do debugowania Xcode na fizycznym urządzeniu</t>
+          <t>VS Code, .NET SDK, Xcode — darmowe narzędzia deweloperskie.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>Mac (kompilacja Xcode)</t>
+          <t>SkiaSharp, SQLite-net, MAUI</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
@@ -2265,185 +2265,131 @@
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>TAK</t>
+          <t>DARMOWE</t>
         </is>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>Wymagany do budowania iOS. Zakładamy że developer ma własny Mac. Jeśli nie — MacBook Air M2 to dodatkowe ~6 000 PLN.</t>
+          <t>Open-source MIT/Apache — zero kosztu, kompatybilne z App Store.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>VS Code / Rider / .NET SDK</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>0 PLN</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
+        <is>
+          <t>SUMA KOSZTÓW STAŁYCH</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>400 PLN/rok</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="inlineStr">
+        <is>
+          <t>Rocznie</t>
+        </is>
+      </c>
+      <c r="D9" s="28" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>Darmowe. Rider ma płatną licencję (opcjonalnie), ale VS Code wystarcza.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>SkiaSharp, SQLite-net, MAUI</t>
-        </is>
-      </c>
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>0 PLN</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D10" s="16" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="E10" s="16" t="inlineStr">
-        <is>
-          <t>Open-source MIT/Apache — darmowe, kompatybilne z App Store</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="28" t="inlineStr">
-        <is>
-          <t>SUMA KOSZTÓW STAŁYCH</t>
-        </is>
-      </c>
-      <c r="B11" s="28" t="inlineStr">
-        <is>
-          <t>5 700 PLN</t>
-        </is>
-      </c>
-      <c r="C11" s="28" t="inlineStr">
-        <is>
-          <t>rok 1</t>
-        </is>
-      </c>
-      <c r="D11" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E11" s="28" t="inlineStr">
-        <is>
-          <t>Przy założeniu posiadanego Maca; bez Maca +6 000 PLN</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="E9" s="28" t="inlineStr">
+        <is>
+          <t>Wyłącznie Apple Developer Account. MacBook i iPady już posiadane — brak zakupów sprzętowych.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>MODEL PRZYCHODÓW — APP STORE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Cena aplikacji (App Store)</t>
+        </is>
+      </c>
+      <c r="B12" s="57" t="inlineStr">
+        <is>
+          <t>Rekomendacja: 49–99 PLN (~12–25 USD)</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Aplikacje medyczno-szkoleniowe na App Store: $9.99–$49.99. Segment B2B (szpitale, uczelnie) akceptuje wyższe ceny.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Prowizja Apple</t>
+        </is>
+      </c>
+      <c r="B13" s="58" t="inlineStr">
+        <is>
+          <t>30% dla nowych deweloperów
+15% gdy przychód &lt; $1M/rok</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Apple Small Business Program: 15% jeśli przychód poniżej $1M. Rejestracja automatyczna.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Cena aplikacji (App Store)</t>
+          <t>Przykład: 100 pobrań × 79 PLN</t>
         </is>
       </c>
       <c r="B14" s="57" t="inlineStr">
         <is>
-          <t>Rekomendacja: 49–99 PLN (~12–25 USD)</t>
+          <t>Przychód brutto: 7 900 PLN
+Po prowizji 15%: ~6 715 PLN</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Aplikacje medyczno-szkoleniowe na App Store: $9.99–$49.99. Segment B2B (szpitale, uczelnie) akceptuje wyższe ceny.</t>
+          <t>Przy 15% prowizji i cenie 79 PLN: zysk ~67 PLN/pobranie. ROI po ~500 pobraniach (33 650 PLN / 67 PLN ≈ 502 pobrania).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Prowizja Apple</t>
+          <t>TestFlight (beta / wgrywanie)</t>
         </is>
       </c>
       <c r="B15" s="58" t="inlineStr">
         <is>
-          <t>30% dla nowych deweloperów
-15% gdy przychód &lt; $1M/rok</t>
+          <t>0 PLN dodatkowych kosztów</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Apple Small Business Program: 15% jeśli przychód poniżej $1M. Rejestracja automatyczna.</t>
+          <t>Wbudowane w Apple Developer Account. Do 10 000 beta testerów. Można używać jako 'dystrybucja do znanych urządzeń' bez App Store.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Przykład: 100 pobrań × 79 PLN</t>
+          <t>Enterprise (znane urządzenia)</t>
         </is>
       </c>
       <c r="B16" s="57" t="inlineStr">
         <is>
-          <t>Przychód brutto: 7 900 PLN
-Po prowizji 15%: ~6 715 PLN</t>
+          <t>1 200 PLN/rok (Apple Developer Enterprise)</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>Przy 15% prowizji i cenie 79 PLN: zysk ~67 PLN/pobranie. ROI po ~500 pobraniach (33 650 PLN / 67 PLN ≈ 502 pobrania).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>TestFlight (beta / wgrywanie)</t>
-        </is>
-      </c>
-      <c r="B17" s="58" t="inlineStr">
-        <is>
-          <t>0 PLN dodatkowych kosztów</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Wbudowane w Apple Developer Account. Do 10 000 beta testerów. Można używać jako 'dystrybucja do znanych urządzeń' bez App Store.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="48" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Enterprise (znane urządzenia)</t>
-        </is>
-      </c>
-      <c r="B18" s="57" t="inlineStr">
-        <is>
-          <t>1 200 PLN/rok (Apple Developer Enterprise)</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Alternatywa: dystrybucja przez MDM bez App Store. Droższe, ale bez ograniczeń App Store review dla zamkniętych instytucji.</t>
         </is>
@@ -2453,11 +2399,11 @@
   <mergeCells count="7">
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="A11:E11"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C12:E12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>